<commit_message>
robust data, self discharging, plot, and simulation adjustments
</commit_message>
<xml_diff>
--- a/Data/Electricity Storage.xlsx
+++ b/Data/Electricity Storage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emirsener/Desktop/Benders-Decomposition/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{603D63B9-AAEB-EE4A-ABD1-C32B0CEAC38A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D1052D-4F5D-3A4C-9CD6-9CB8BCD7ADFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
   <si>
     <t>Metrics</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t>Discharging efficiency</t>
+  </si>
+  <si>
+    <t>Self discharge rate</t>
   </si>
 </sst>
 </file>
@@ -464,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5344E307-70EA-9749-BC3D-54A83804696F}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.33203125" bestFit="1" customWidth="1"/>
@@ -572,6 +575,15 @@
       </c>
       <c r="B12">
         <v>0.9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13">
+        <f>1-0.0006</f>
+        <v>0.99939999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
simulation, env, and robust data adjs.
</commit_message>
<xml_diff>
--- a/Data/Electricity Storage.xlsx
+++ b/Data/Electricity Storage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emirsener/Desktop/Benders-Decomposition/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D1052D-4F5D-3A4C-9CD6-9CB8BCD7ADFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5615014-8346-2D48-B1AE-7D7D4F455307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
   </bookViews>
@@ -486,8 +486,8 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <f>350*1000/0.9</f>
-        <v>388888.88888888888</v>
+        <f>275*1000/0.9</f>
+        <v>305555.55555555556</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -513,7 +513,8 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <f>275*1000*0.02</f>
+        <v>5500</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>

</xml_diff>

<commit_message>
decision tree plot adj
</commit_message>
<xml_diff>
--- a/Data/Electricity Storage.xlsx
+++ b/Data/Electricity Storage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emirsener/Desktop/Benders-Decomposition/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B82296-E0D5-DF40-8FF2-A90C47B2ABD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A8B0345-8B99-3349-9150-5428FD325F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20000" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
+    <workbookView xWindow="20" yWindow="680" windowWidth="34560" windowHeight="20000" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
   </bookViews>
   <sheets>
     <sheet name="Initial values" sheetId="7" r:id="rId1"/>
@@ -513,8 +513,8 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <f>275*10000*0.02</f>
-        <v>55000</v>
+        <f>ROUND(275*10000*0.02/0.9,0)</f>
+        <v>61111</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -542,8 +542,8 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <f>ROUND(0.03*10000/0.9,4)</f>
-        <v>333.33330000000001</v>
+        <f>ROUND(0.03*10000/0.9,1)</f>
+        <v>333.3</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
emission, monte carlo adjustments
</commit_message>
<xml_diff>
--- a/Data/Electricity Storage.xlsx
+++ b/Data/Electricity Storage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emirsener/Desktop/Benders-Decomposition/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A8B0345-8B99-3349-9150-5428FD325F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E890545F-D0C8-0E47-9BFB-9016EE42AAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="680" windowWidth="34560" windowHeight="20000" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20000" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
   </bookViews>
   <sheets>
     <sheet name="Initial values" sheetId="7" r:id="rId1"/>
@@ -513,8 +513,8 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <f>ROUND(275*10000*0.02/0.9,0)</f>
-        <v>61111</v>
+        <f>ROUND(275*10000*0.02,0)</f>
+        <v>55000</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -542,8 +542,8 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <f>ROUND(0.03*10000/0.9,1)</f>
-        <v>333.3</v>
+        <f>ROUND(0.03*10000,1)</f>
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>